<commit_message>
New update on file
</commit_message>
<xml_diff>
--- a/12515872.xlsx
+++ b/12515872.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MSC IT\Msc IT sem 3\PROGRAMMING IN PYTHON\CAP776\CAP-776\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\MSC IT\Msc IT sem 3\PROGRAMMING IN PYTHON\CAP776\CAP-776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC3FAAE-DED1-48FC-93E6-C4E6CB81B7E6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A6308B-6875-40AB-9B98-F84FEAF7CE19}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10110" windowHeight="4380" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,24 @@
   </si>
   <si>
     <t>tired afterclasses</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Had a good day</t>
+  </si>
+  <si>
+    <t>longest fitness time</t>
+  </si>
+  <si>
+    <t>fitness was good today</t>
+  </si>
+  <si>
+    <t>Learn a lot today at school</t>
   </si>
 </sst>
 </file>
@@ -1538,109 +1556,219 @@
       <c r="E17" s="14">
         <v>90</v>
       </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
+      <c r="F17" s="14">
+        <v>360</v>
+      </c>
+      <c r="G17" s="14">
+        <v>6</v>
+      </c>
+      <c r="H17" s="14">
+        <v>120</v>
+      </c>
       <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v>650</v>
+        <v>1130</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v>790</v>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
+        <v>310</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="13">
+        <v>46255</v>
+      </c>
+      <c r="B18" s="14">
+        <v>420</v>
+      </c>
+      <c r="C18" s="14">
+        <v>90</v>
+      </c>
+      <c r="D18" s="14">
+        <v>60</v>
+      </c>
+      <c r="E18" s="14">
+        <v>90</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14">
+        <v>120</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>780</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>660</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B19" s="14">
+        <v>420</v>
+      </c>
+      <c r="C19" s="14">
+        <v>60</v>
+      </c>
+      <c r="D19" s="14">
+        <v>60</v>
+      </c>
+      <c r="E19" s="14">
+        <v>0</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14">
+        <v>0</v>
+      </c>
+      <c r="H19" s="14">
+        <v>0</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>540</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>900</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B20" s="14">
+        <v>420</v>
+      </c>
+      <c r="C20" s="14">
+        <v>60</v>
+      </c>
+      <c r="D20" s="14">
+        <v>90</v>
+      </c>
+      <c r="E20" s="14">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14">
+        <v>0</v>
+      </c>
+      <c r="H20" s="14">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>570</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>870</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B21" s="14">
+        <v>270</v>
+      </c>
+      <c r="C21" s="14">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14">
+        <v>180</v>
+      </c>
+      <c r="E21" s="14">
+        <v>120</v>
+      </c>
+      <c r="F21" s="14">
+        <v>360</v>
+      </c>
+      <c r="G21" s="14">
+        <v>6</v>
+      </c>
+      <c r="H21" s="14">
+        <v>120</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>

</xml_diff>